<commit_message>
Keep workflow decisions and tables readable across report sizes
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R26e096f09f5547e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R87f9c11fb66b4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R6d273cc3bf714baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rbc2183514cd54a8d"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Identify sample input separately from custom report data
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R6d273cc3bf714baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rbc2183514cd54a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rbbfd951f8e6a4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R4e70e627a2954eaf"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Reject ambiguous amounts in budget forecast inputs
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rbbfd951f8e6a4dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R4e70e627a2954eaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R820ca2c0a8ac4c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rb40f008f96614ba2"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Record PowerShell showcase generation provenance
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R820ca2c0a8ac4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rb40f008f96614ba2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R736b0aeff6954b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R948045ec81394716"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Preserve exact showcase source bytes across checkouts
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R736b0aeff6954b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R948045ec81394716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rc7d373926cd5425a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R3571a40a9bc44b07"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Bind showcase evidence to its executable producer
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rc7d373926cd5425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R3571a40a9bc44b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Ra25d2a8e7b4f42c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R9afa78e2febb4a1b"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Validate complete showcase receipts and separate preview review
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Ra25d2a8e7b4f42c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R9afa78e2febb4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rf0cff7949c2e485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rce0dec04d81e4adb"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Bind showcase builder and run child evidence contracts in CI
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rf0cff7949c2e485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rce0dec04d81e4adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R548468e667654ca0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R3b6290dd5c424454"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Run workflow examples with installed modules and downloaded CSV inputs
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R548468e667654ca0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R3b6290dd5c424454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Ref91ddb81513449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R274c9815db274e22"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Complete integrated documentation and release validation paths
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Ref91ddb81513449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R274c9815db274e22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7a75d10e867d49d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R0e190eb094354913"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh PSWriteOffice 3.5.2 website showcase evidence
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7a75d10e867d49d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R0e190eb094354913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R10c8d8703c384725"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra8ea42c30f224549"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh PSWriteOffice 3.5.2 website showcase evidence (#3182)
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7a75d10e867d49d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R0e190eb094354913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R10c8d8703c384725"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra8ea42c30f224549"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh the website examples and their generation evidence
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R10c8d8703c384725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra8ea42c30f224549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R3d35d32bce774692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R64f0182efde14ef8"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>
@@ -128,12 +128,12 @@
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
   <x:fills count="3">
@@ -200,6 +200,289 @@
 </x:table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="OfficeIMO Modern">
+  <a:themeElements>
+    <a:clrScheme name="Modern">
+      <a:dk1>
+        <a:srgbClr val="1B2433"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="5B6575"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="F6F8FB"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="3F64D7"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="DC7536"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="058E80"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="A52758"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="3F2F6B"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="255319"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="3F64D7"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="A52758"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Modern">
+      <a:majorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>

</xml_diff>

<commit_message>
Refresh Word text help and executable examples
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R3d35d32bce774692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R64f0182efde14ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7c1db81b866e4b84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R55bd6817ef724d7c"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh PowerShell website artifacts and runnable showcases
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7c1db81b866e4b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R55bd6817ef724d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R77f1540e2cb048fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra0c320693b9044c3"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh module help and website examples from the current API
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R77f1540e2cb048fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra0c320693b9044c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R23d516758178410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rb5db0b646ead4859"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh command documentation and current API links
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R23d516758178410f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rb5db0b646ead4859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R0f93341d129e4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R91c89b9e8c3949f9"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh generated command evidence and source links
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R0f93341d129e4a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R91c89b9e8c3949f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rad90a4fca023407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R9e33e90def3e41e3"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh shared image documentation and conversion routes
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rad90a4fca023407e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R9e33e90def3e41e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R9991f8597c95488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rae755110e1b44b40"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh packaged command evidence and source references
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R9991f8597c95488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Rae755110e1b44b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rf12fe6a64e354bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Racecc73ab12e4587"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh PowerShell showcase and API evidence for version 3.5.3
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R10c8d8703c384725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra8ea42c30f224549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R3b34922c4ba44b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R595d3c33ea674765"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Refresh qualified command help and executed PowerShell showcases
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rf12fe6a64e354bfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Racecc73ab12e4587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R7378c2bba3834b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R9da7abd2a946410a"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>

<commit_message>
Expand Excel formula support and reduce lookup allocations (#3227)
Calculate composed lookup fallbacks and dependent totals, expand lookup, reference, array and named-expression support, and preserve native blank and typed-error behavior. Reduce formula allocation through shared-string snapshots, lazy lookup sources and per-pass name catalogs.

Validate native Excel values and spills, supported targets and equivalent report and binary-search workloads.

Fixes #3226.
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
+++ b/Website/static/downloads/showcase/pswriteoffice/budget-forecast-review.xlsx
@@ -5,8 +5,8 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R10c8d8703c384725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="Ra8ea42c30f224549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R3b34922c4ba44b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail" sheetId="2" r:id="R595d3c33ea674765"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Review'!$A$1:$B$8</x:definedName>

</xml_diff>